<commit_message>
Programme juin - juillet 2026
</commit_message>
<xml_diff>
--- a/outils/work/tableau_ingest.xlsx
+++ b/outils/work/tableau_ingest.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Sukkwan island</t>
+          <t>Father</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -472,7 +472,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>mercredi 13 mai</t>
+          <t>mercredi 10 juin</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -484,17 +484,13 @@
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>La fille du Kombini</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>L'abandon</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>jeudi 14 mai</t>
+          <t>jeudi 11 juin</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -506,43 +502,43 @@
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Nous l'orchestre</t>
+          <t>Minuscule - La vallée des fourmis perdues - SCOL</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>vendredi 15 mai</t>
+          <t>vendredi 12 juin</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>10h</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Jeune pousse</t>
+          <t>Zootopia 2 - SCOL</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>samedi 16 mai</t>
+          <t>vendredi 12 juin</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>17h</t>
+          <t>14h</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Good luck have fun don't die</t>
+          <t>L'être aimé</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -552,101 +548,101 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>samedi 16 mai</t>
+          <t>vendredi 12 juin</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Mauvaise pioche</t>
+          <t>L'odyssée de Céleste</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>samedi 16 mai</t>
+          <t>dimanche 14 juin</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>16h</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>L'odyssée de Céleste</t>
+          <t>Histoires parralèles</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>dimanche 17 mai</t>
+          <t>dimanche 14 juin</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Juste une illusion</t>
+          <t>Tout va super</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>dimanche 17 mai</t>
+          <t>dimanche 14 juin</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Au fil de l'eau - SCOL</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
+          <t>The new west</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>mardi 19 mai</t>
+          <t>mardi 16 juin</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>10h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Sorda</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>L'affaire Zanetti</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>mardi 19 mai</t>
+          <t>mercredi 17 juin</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -658,17 +654,13 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>La corde au cou</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Histoires parralèles</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>mercredi 20 mai</t>
+          <t>jeudi 18 juin</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -680,31 +672,31 @@
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Mi amor</t>
+          <t>Tout en haut du monde - SCOL</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>jeudi 21 mai</t>
+          <t>vendredi 19 juin</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>9h30</t>
         </is>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Compostelle</t>
+          <t>Pour le plaisir</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>vendredi 22 mai</t>
+          <t>vendredi 19 juin</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -716,7 +708,7 @@
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Mon grand frère et moi</t>
+          <t>Le garçon qui faisait danser les collines</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -726,7 +718,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>vendredi 22 mai</t>
+          <t>vendredi 19 juin</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -738,25 +730,25 @@
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Super Mario Galaxy Le film</t>
+          <t>Nouveaux copains à Puffin Rock</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>samedi 23 mai</t>
+          <t>samedi 20 juin</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>16h30</t>
         </is>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Nuestra tierra</t>
+          <t>Star wars The Mandalorian and Grogu</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -766,7 +758,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>samedi 23 mai</t>
+          <t>samedi 20 juin</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -778,17 +770,13 @@
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Michaël</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>L'abandon</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>samedi 23 mai</t>
+          <t>samedi 20 juin</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -800,13 +788,13 @@
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Le secret du loup d'Ethiopie</t>
+          <t>CHaO</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>dimanche 24 mai</t>
+          <t>dimanche 21 juin</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -818,13 +806,13 @@
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>C'est quoi l'amour ?</t>
+          <t>Autofiction</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>dimanche 24 mai</t>
+          <t>dimanche 21 juin</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -836,191 +824,183 @@
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Le cri des gardes</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Rencontres vidéos scolaires</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>dimanche 24 mai</t>
+          <t>mardi 23 juin</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>9h30</t>
         </is>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>L'enfant du désert</t>
+          <t>La vénus électrique</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>lundi 25 mai</t>
+          <t>mardi 23 juin</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>17h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>MacPat le chat chanteur - SCOL</t>
+          <t>L'être aimé</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>mardi 26 mai</t>
+          <t>mercredi 24 juin</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>10h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Dans la roue du petit Prince - SCOL</t>
+          <t>D'un monde à l'autre</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>mardi 26 mai</t>
+          <t>jeudi 25 juin</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>14h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Projet dernière chance</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>C'est quoi l'amour ?</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>mardi 26 mai</t>
+          <t>vendredi 26 juin</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>20h30</t>
+          <t>15h</t>
         </is>
       </c>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>Conférence filmée Serge Tisseron</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
+          <t>Colony</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>mercredi 27 mai</t>
+          <t>vendredi 26 juin</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>18h30</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>The world of love</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Super Mario Galaxy Le film</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>mercredi 27 mai</t>
+          <t>dimanche 28 juin</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>16h</t>
         </is>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>Soumsoum la nuit des astres</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>L'objet du délit</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>jeudi 28 mai</t>
+          <t>dimanche 28 juin</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Bily Elliot - SCOL</t>
+          <t>Le vertige</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>vendredi 29 mai</t>
+          <t>dimanche 28 juin</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>9h30</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>Juste une illusion</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
+          <t>The Christophers</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>vendredi 29 mai</t>
+          <t>mardi 30 juin</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1032,93 +1012,89 @@
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>Elfie et les supers Elfkins</t>
+          <t>Sur la route d'Omaha</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>dimanche 31 mai</t>
+          <t>mercredi 1 juillet</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="32" ht="40" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>Pour le meilleur</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
+          <t>Autofiction</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>dimanche 31 mai</t>
+          <t>vendredi 3 juillet</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="33" ht="40" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>Elise sous emprise</t>
+          <t>Nouveaux copains à Puffin Rock</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>dimanche 31 mai</t>
+          <t>samedi 4 juillet</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>16h30</t>
         </is>
       </c>
     </row>
     <row r="34" ht="40" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Hayat</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Star wars The Mandalorian and Grogu</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>mardi 2 juin</t>
+          <t>samedi 4 juillet</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>20h30</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>Romeria</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La bataille de Gaulle L'âge de fer</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>mercredi 3 juin</t>
+          <t>samedi 4 juillet</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1130,17 +1106,13 @@
     <row r="36" ht="40" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>Cocotte</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Ulysse</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>jeudi 4 juin</t>
+          <t>dimanche 5 juillet</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1152,168 +1124,38 @@
     <row r="37" ht="40" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>La vénus électrique</t>
+          <t>Scarlet et l'éternité</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>vendredi 5 juin</t>
+          <t>mardi 7 juillet</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>16h</t>
         </is>
       </c>
     </row>
     <row r="38" ht="40" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>L'odyssée de Céleste JP</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
+          <t>L'illusion de Yakushima</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>samedi 6 juin</t>
+          <t>mardi 7 juillet</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>16h</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="40" customHeight="1">
-      <c r="A39" s="1" t="inlineStr">
-        <is>
-          <t>Vol au-dessus d'un nid de coucou</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>samedi 6 juin</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>18h</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="40" customHeight="1">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>Le diable s'habille en Prada 2</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>samedi 6 juin</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="40" customHeight="1">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>ChaO</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>dimanche 7 juin</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>16h</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="40" customHeight="1">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t>La vénus électrique</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>dimanche 7 juin</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>18h</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="40" customHeight="1">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>Contes sur moi - SCOL</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr"/>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>lundi 8 juin</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>10h</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="40" customHeight="1">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t>Le roi des masques - SCOL</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>mardi 9 juin</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>10h</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="40" customHeight="1">
-      <c r="A45" s="1" t="inlineStr">
-        <is>
-          <t>Vivaldi et moi</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>mardi 9 juin</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>21h</t>
         </is>

</xml_diff>

<commit_message>
Mettre a jour programme et prochainement
</commit_message>
<xml_diff>
--- a/outils/work/tableau_ingest.xlsx
+++ b/outils/work/tableau_ingest.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Father</t>
+          <t>The plague</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>mercredi 10 juin</t>
+          <t>mercredi 8 juillet</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -502,67 +502,79 @@
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>L'abandon</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr"/>
+          <t>Le dernier souffle d'un yakusa</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>jeudi 11 juin</t>
+          <t>jeudi 9 juillet</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Minuscule - SCOL</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr"/>
+          <t>Disclosure day</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>vendredi 12 juin</t>
+          <t>jeudi 9 juillet</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>10h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Zootopia 2 - SCOL</t>
+          <t>Juste une illusion</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>vendredi 12 juin</t>
+          <t>vendredi 10 juillet</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>14h</t>
+          <t>15h</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>L'être aimé</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
+          <t>Seuls les rebelles</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>vendredi 12 juin</t>
+          <t>vendredi 10 juillet</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -574,13 +586,13 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>L'odyssée de Céleste</t>
+          <t>James et la pêche géante</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>dimanche 14 juin</t>
+          <t>samedi 11 juillet</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -592,13 +604,13 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Histoires parralèles</t>
+          <t>La baleine et le musicien</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr"/>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>dimanche 14 juin</t>
+          <t>samedi 11 juillet</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -610,13 +622,17 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Tout va super</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr"/>
+          <t>Le virtuose</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>dimanche 14 juin</t>
+          <t>samedi 11 juillet</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -628,35 +644,31 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>The new west</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La bataille de Gaulle L'âge de fer</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>mardi 16 juin</t>
+          <t>dimanche 12 juillet</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h30</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>L'affaire Zanetti</t>
+          <t>L'étrangère</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr"/>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>mercredi 17 juin</t>
+          <t>mardi 14 juillet</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -668,101 +680,97 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Histoires parralèles</t>
+          <t>Toy story 5</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>jeudi 18 juin</t>
+          <t>jeudi 16 juillet</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Tout en haut du monde - SCOL</t>
+          <t>In waves</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr"/>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>vendredi 19 juin</t>
+          <t>jeudi 16 juillet</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>9h30</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Pour le plaisir</t>
+          <t>Disclosure day</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr"/>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>vendredi 19 juin</t>
+          <t>vendredi 17 juillet</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Le garçon qui faisait danser les collines</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Un champ de fraises pour l’éternité</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>vendredi 19 juin</t>
+          <t>dimanche 19 juillet</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Nouveaux copains à Puffin Rock</t>
+          <t>Les beaux jours</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr"/>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>samedi 20 juin</t>
+          <t>mardi 21 juillet</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>16h30</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Star wars The Mandalorian and Grogu</t>
+          <t>Notre histoire - Chroniques du Caire</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -772,123 +780,115 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>samedi 20 juin</t>
+          <t>mardi 21 juillet</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>L'abandon</t>
+          <t>Entre ciel et terre</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>samedi 20 juin</t>
+          <t>jeudi 23 juillet</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>CHaO</t>
+          <t>L’écologie des sentiments</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>dimanche 21 juin</t>
+          <t>jeudi 23 juillet</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Autofiction</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La bataille de Gaulle Partie 2 J'écris ton nom</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>dimanche 21 juin</t>
+          <t>vendredi 24 juillet</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Rencontres vidéos scolaires</t>
+          <t>Les Parfait(s) Arnaques en famillre</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>mardi 23 juin</t>
+          <t>dimanche 26 juillet</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>9h30</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>La vénus électrique</t>
+          <t>Toy story 5</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr"/>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>mardi 23 juin</t>
+          <t>mardi 28 juillet</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>L'être aimé</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La chaleur</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>mercredi 24 juin</t>
+          <t>mardi 28 juillet</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -900,53 +900,53 @@
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>D'un monde à l'autre</t>
+          <t>Des minions et des monstres</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>jeudi 25 juin</t>
+          <t>jeudi 30 juillet</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>C'est quoi l'amour ?</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr"/>
+          <t>D'où vient le vent</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>vendredi 26 juin</t>
+          <t>jeudi 30 juillet</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Colony</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>On l'appelait Robin des Bois</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr"/>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>vendredi 26 juin</t>
+          <t>vendredi 31 juillet</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -958,230 +958,56 @@
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Super Mario Galaxy Le film</t>
+          <t>La bataille de Gaulle Partie 2 J'écris ton nom</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>dimanche 28 juin</t>
+          <t>dimanche 2 aout</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>17h30</t>
         </is>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>L'objet du délit</t>
+          <t>Kayara, princesse inca</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>dimanche 28 juin</t>
+          <t>mardi 4 aout</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Le vertige</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr"/>
+          <t>The last viking</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>dimanche 28 juin</t>
+          <t>mardi 4 aout</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>The Christophers</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>mardi 30 juin</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Sur la route d'Omaha</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>mercredi 1 juillet</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Autofiction</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>vendredi 3 juillet</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="40" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Nouveaux copains à Puffin Rock</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>samedi 4 juillet</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>16h30</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="40" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Star wars The Mandalorian and Grogu</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>samedi 4 juillet</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>18h</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>La bataille de Gaulle L'âge de fer</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>samedi 4 juillet</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="40" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Ulysse</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr"/>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>dimanche 5 juillet</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="40" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Scarlet et l'éternité</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>mardi 7 juillet</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>16h</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>L'illusion de Yakushima</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>mardi 7 juillet</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>21h</t>
         </is>

</xml_diff>

<commit_message>
modif a bras le corps
</commit_message>
<xml_diff>
--- a/outils/work/tableau_ingest.xlsx
+++ b/outils/work/tableau_ingest.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Father</t>
+          <t>The plague</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>mercredi 10 juin</t>
+          <t>mercredi 8 juillet</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -502,67 +502,79 @@
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>L'abandon</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr"/>
+          <t>Le dernier souffle d'un yakusa</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>jeudi 11 juin</t>
+          <t>jeudi 9 juillet</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Minuscule - SCOL</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr"/>
+          <t>Disclosure day</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>vendredi 12 juin</t>
+          <t>jeudi 9 juillet</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>10h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Zootopia 2 - SCOL</t>
+          <t>Juste une illusion</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>vendredi 12 juin</t>
+          <t>vendredi 10 juillet</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>14h</t>
+          <t>15h</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>L'être aimé</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
+          <t>Seuls les rebelles</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>vendredi 12 juin</t>
+          <t>vendredi 10 juillet</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -574,13 +586,13 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>L'odyssée de Céleste</t>
+          <t>James et la pêche géante</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>dimanche 14 juin</t>
+          <t>samedi 11 juillet</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -592,13 +604,13 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Histoires parralèles</t>
+          <t>La baleine et le musicien</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr"/>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>dimanche 14 juin</t>
+          <t>samedi 11 juillet</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -610,13 +622,17 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Tout va super</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr"/>
+          <t>Le virtuose</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>dimanche 14 juin</t>
+          <t>samedi 11 juillet</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -628,35 +644,31 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>The new west</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La bataille de Gaulle L'âge de fer</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>mardi 16 juin</t>
+          <t>dimanche 12 juillet</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h30</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>L'affaire Zanetti</t>
+          <t>L'étrangère</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr"/>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>mercredi 17 juin</t>
+          <t>mardi 14 juillet</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -668,101 +680,97 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Histoires parralèles</t>
+          <t>Toy story 5</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>jeudi 18 juin</t>
+          <t>jeudi 16 juillet</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Tout en haut du monde - SCOL</t>
+          <t>In waves</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr"/>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>vendredi 19 juin</t>
+          <t>jeudi 16 juillet</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>9h30</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Pour le plaisir</t>
+          <t>Disclosure day</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr"/>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>vendredi 19 juin</t>
+          <t>vendredi 17 juillet</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Le garçon qui faisait danser les collines</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>Un champ de fraises pour l’éternité</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>vendredi 19 juin</t>
+          <t>dimanche 19 juillet</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Nouveaux copains à Puffin Rock</t>
+          <t>Les beaux jours</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr"/>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>samedi 20 juin</t>
+          <t>mardi 21 juillet</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>16h30</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Star wars The Mandalorian and Grogu</t>
+          <t>Notre histoire - Chroniques du Caire</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -772,123 +780,115 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>samedi 20 juin</t>
+          <t>mardi 21 juillet</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>L'abandon</t>
+          <t>Entre ciel et terre</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>samedi 20 juin</t>
+          <t>jeudi 23 juillet</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>CHaO</t>
+          <t>L’écologie des sentiments</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>dimanche 21 juin</t>
+          <t>jeudi 23 juillet</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Autofiction</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La bataille de Gaulle Partie 2 J'écris ton nom</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>dimanche 21 juin</t>
+          <t>vendredi 24 juillet</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Rencontres vidéos scolaires</t>
+          <t>Les Parfait(s) Arnaques en famillre</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>mardi 23 juin</t>
+          <t>dimanche 26 juillet</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>9h30</t>
+          <t>18h</t>
         </is>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>La vénus électrique</t>
+          <t>Toy story 5</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr"/>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>mardi 23 juin</t>
+          <t>mardi 28 juillet</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>L'être aimé</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>La chaleur</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>mercredi 24 juin</t>
+          <t>mardi 28 juillet</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -900,53 +900,53 @@
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>D'un monde à l'autre</t>
+          <t>Des minions et des monstres</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>jeudi 25 juin</t>
+          <t>jeudi 30 juillet</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>C'est quoi l'amour ?</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr"/>
+          <t>D'où vient le vent</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>vendredi 26 juin</t>
+          <t>jeudi 30 juillet</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>21h</t>
         </is>
       </c>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Colony</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
+          <t>On l'appelait Robin des Bois</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr"/>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>vendredi 26 juin</t>
+          <t>vendredi 31 juillet</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -958,230 +958,56 @@
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Super Mario Galaxy Le film</t>
+          <t>La bataille de Gaulle Partie 2 J'écris ton nom</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>dimanche 28 juin</t>
+          <t>dimanche 2 aout</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>16h</t>
+          <t>17h30</t>
         </is>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>L'objet du délit</t>
+          <t>Kayara, princesse inca</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>dimanche 28 juin</t>
+          <t>mardi 4 aout</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>17h</t>
         </is>
       </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Le vertige</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr"/>
+          <t>The last viking</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>dimanche 28 juin</t>
+          <t>mardi 4 aout</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>The Christophers</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>mardi 30 juin</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Sur la route d'Omaha</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>mercredi 1 juillet</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Autofiction</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>vendredi 3 juillet</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="40" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Nouveaux copains à Puffin Rock</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>samedi 4 juillet</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>16h30</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="40" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Star wars The Mandalorian and Grogu</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>samedi 4 juillet</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>18h</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>La bataille de Gaulle L'âge de fer</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>samedi 4 juillet</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="40" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Ulysse</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr"/>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>dimanche 5 juillet</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>21h</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="40" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Scarlet et l'éternité</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>mardi 7 juillet</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>16h</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>L'illusion de Yakushima</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>mardi 7 juillet</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>21h</t>
         </is>

</xml_diff>